<commit_message>
creating complete data files 2005
</commit_message>
<xml_diff>
--- a/notebooks/2005_Birth/01_missing_values.xlsx
+++ b/notebooks/2005_Birth/01_missing_values.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -522,7 +522,7 @@
         <v>9</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>370652</v>
+        <v>370646</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>100</v>
@@ -549,7 +549,7 @@
         <v>12</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>370707</v>
+        <v>370701</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>100</v>
@@ -576,7 +576,7 @@
         <v>25</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>370731</v>
+        <v>370725</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>100</v>
@@ -585,7 +585,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Registered_Month</t>
+          <t>Birh_Year 2.0</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
@@ -596,14 +596,14 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>370731</v>
+        <v>370725</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>100</v>
@@ -630,7 +630,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>370731</v>
+        <v>370725</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>100</v>
@@ -639,7 +639,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Birth_Month</t>
+          <t>Registered_Month</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
@@ -657,7 +657,7 @@
         <v>12</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>370731</v>
+        <v>370725</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>100</v>
@@ -666,7 +666,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Birh_Year</t>
+          <t>Birth_Month</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
@@ -677,14 +677,14 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>64</v>
+        <v>12</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>370731</v>
+        <v>370725</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>100</v>
@@ -693,7 +693,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Hospital or Not</t>
+          <t>Birh_Year</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
@@ -704,14 +704,14 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>370731</v>
+        <v>370725</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>100</v>
@@ -720,7 +720,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Gender</t>
+          <t>Hospital or Not</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
@@ -738,7 +738,7 @@
         <v>2</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>370731</v>
+        <v>370725</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>100</v>
@@ -747,7 +747,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>BORDER</t>
+          <t>Gender</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
@@ -758,14 +758,14 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>370731</v>
+        <v>370725</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>100</v>
@@ -774,7 +774,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Age of Mother</t>
+          <t>BORDER</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
@@ -789,10 +789,10 @@
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>41</v>
+        <v>13</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>370731</v>
+        <v>370725</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>100</v>
@@ -801,7 +801,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Marital_Status</t>
+          <t>Age of Mother</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
@@ -812,14 +812,14 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>370731</v>
+        <v>370725</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>100</v>
@@ -828,27 +828,54 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>Marital_Status</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>370725</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>District_of_Mother</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>str</t>
         </is>
       </c>
-      <c r="E14" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="F14" s="3" t="n">
-        <v>370731</v>
-      </c>
-      <c r="G14" s="3" t="n">
+      <c r="E15" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>370725</v>
+      </c>
+      <c r="G15" s="3" t="n">
         <v>100</v>
       </c>
     </row>
@@ -889,7 +916,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>370731</v>
+        <v>370725</v>
       </c>
     </row>
     <row r="3">
@@ -899,7 +926,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">

</xml_diff>